<commit_message>
Blindar importación Excel anti duplicados
Co-authored-by: aulamasia-droid <242687825+aulamasia-droid@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/Plantilla_Ecometrics_IRM.xlsx
+++ b/public/Plantilla_Ecometrics_IRM.xlsx
@@ -668,7 +668,8 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -717,7 +718,7 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>⚠  Usa los menús desplegables en columnas MATERIAL y CLIENTE.  La FECHA debe corresponder al mes del período seleccionado en Ecometrics.</t>
+          <t>⚠ Usa los menús desplegables en MATERIAL y CLIENTE. La FECHA debe corresponder al mes seleccionado. Si cuentas con IMPORTE PAGADO, llénalo para que Ecometrics calcule el impacto económico exacto.</t>
         </is>
       </c>
     </row>
@@ -745,6 +746,16 @@
       <c r="E5" s="9" t="inlineStr">
         <is>
           <t>NOTAS</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>PRECIO</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>IMPORTE PAGADO</t>
         </is>
       </c>
     </row>
@@ -4296,7 +4307,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4615,7 +4626,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="C4AE"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>